<commit_message>
Rev4 order package: add lead-time / sourcing column and README section for the short and low lines
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqGG2zxwCtVNzoezLoNxXN
</commit_message>
<xml_diff>
--- a/rev4/order/Rev4_JLCPCB_Order.xlsx
+++ b/rev4/order/Rev4_JLCPCB_Order.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="319">
   <si>
     <t xml:space="preserve">Comment</t>
   </si>
@@ -717,6 +717,9 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
+    <t xml:space="preserve">Lead time / sourcing</t>
+  </si>
+  <si>
     <t xml:space="preserve">CL10B104KA8NNNC</t>
   </si>
   <si>
@@ -732,6 +735,9 @@
     <t xml:space="preserve">optional Basic swap: CC0603KRX7R9BB104 100nF 50V X7R (saves one Extended fee)</t>
   </si>
   <si>
+    <t xml:space="preserve">In stock at JLCPCB: no part lead time; only the PCBA lead time applies.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CL10B474KA8NNNC</t>
   </si>
   <si>
@@ -786,6 +792,9 @@
     <t xml:space="preserve">optional: 1N5819WS SOD-323 40V 1A, Basic, 4.4M stock — drop-in for D1 if NSR1020MW2T3G runs short (501 in stock)</t>
   </si>
   <si>
+    <t xml:space="preserve">In stock at JLCPCB (501, 1 per board): no part lead time for runs up to ~450 boards after attrition. Beyond stock: global sourcing 9-20 business days, or Basic drop-in C191023 (4.4M pcs).</t>
+  </si>
+  <si>
     <t xml:space="preserve">1N5817W</t>
   </si>
   <si>
@@ -804,6 +813,9 @@
     <t xml:space="preserve">SOFNG</t>
   </si>
   <si>
+    <t xml:space="preserve">In stock at JLCPCB (1,407): no part lead time. Beyond stock: global sourcing 9-20 business days.</t>
+  </si>
+  <si>
     <t xml:space="preserve">DFE201610P-2R2M=P2</t>
   </si>
   <si>
@@ -939,6 +951,9 @@
     <t xml:space="preserve">YTL</t>
   </si>
   <si>
+    <t xml:space="preserve">In stock at JLCPCB (1,850): no part lead time. Beyond stock: global sourcing 9-20 business days.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TPA6110A2DGNR</t>
   </si>
   <si>
@@ -951,6 +966,9 @@
     <t xml:space="preserve">CRITICAL: 5 in stock, min buy 7. TPA6111A2DR (C497472, 887 in stock) is SOIC-8, not the HVSSOP-8-EP footprint; TPA6111A2DGN(R) HVSSOP parts show 0 stock. Options: buy TPA6110A2DGNR from Mouser/Digi-Key and consign or hand-solder U3; or JLC global-sourcing pre-order (lead time); or change U3 to SOIC-8 on the next spin</t>
   </si>
   <si>
+    <t xml:space="preserve">SHORT at JLCPCB (5 pcs, min buy 7; LCSC 5 pcs, pre-sale flagged; TI store: out of stock; lifecycle ACTIVE). Fastest: Digi-Key (~528 pcs) or Mouser (~2,165 pcs, aggregator snapshot, verify live) ship in-stock parts in 1-3 days + transit, then hand-solder or consign. JLCPCB global sourcing: 1-3 business days review + 9-20 business days, assembly waits for arrival. JLCPCB pre-order: no lead time published.</t>
+  </si>
+  <si>
     <t xml:space="preserve">MAX9814ETD+T</t>
   </si>
   <si>
@@ -958,6 +976,9 @@
   </si>
   <si>
     <t xml:space="preserve">TPS62172DSGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In stock at JLCPCB (1,993): no part lead time. Beyond stock: global sourcing 9-20 business days.</t>
   </si>
 </sst>
 </file>
@@ -2455,7 +2476,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2469,7 +2490,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2523,16 +2544,19 @@
       <c r="M3" s="1" t="s">
         <v>230</v>
       </c>
+      <c r="N3" s="1" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>6</v>
@@ -2551,7 +2575,7 @@
         <v>1696733</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.0143</v>
@@ -2561,10 +2585,13 @@
         <v>OK</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2572,10 +2599,10 @@
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>6</v>
@@ -2594,7 +2621,7 @@
         <v>836122</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.0297</v>
@@ -2605,16 +2632,19 @@
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
+      <c r="N5" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
@@ -2633,7 +2663,7 @@
         <v>54269</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>0.0384</v>
@@ -2644,16 +2674,19 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
+      <c r="N6" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>6</v>
@@ -2672,7 +2705,7 @@
         <v>170136</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.0199</v>
@@ -2682,10 +2715,13 @@
         <v>OK</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2693,10 +2729,10 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>6</v>
@@ -2715,7 +2751,7 @@
         <v>1803414</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.0131</v>
@@ -2725,10 +2761,13 @@
         <v>OK</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2736,10 +2775,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>6</v>
@@ -2758,7 +2797,7 @@
         <v>6247019</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.0101</v>
@@ -2769,16 +2808,19 @@
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
+      <c r="N9" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>26</v>
@@ -2797,7 +2839,7 @@
         <v>3999370</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.0689</v>
@@ -2808,16 +2850,19 @@
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
+      <c r="N10" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>26</v>
@@ -2836,7 +2881,7 @@
         <v>3483126</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.2372</v>
@@ -2847,16 +2892,19 @@
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N11" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>33</v>
@@ -2875,7 +2923,7 @@
         <v>501</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.2814</v>
@@ -2885,10 +2933,13 @@
         <v>OK</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2896,10 +2947,10 @@
         <v>38</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>37</v>
@@ -2918,7 +2969,7 @@
         <v>3587</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.0199</v>
@@ -2929,16 +2980,19 @@
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
+      <c r="N13" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>6</v>
@@ -2957,7 +3011,7 @@
         <v>1361603</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.0146</v>
@@ -2968,16 +3022,19 @@
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N14" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>44</v>
@@ -2996,7 +3053,7 @@
         <v>1407</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.2909</v>
@@ -3007,19 +3064,22 @@
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
+      <c r="N15" s="2" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>257</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>47</v>
@@ -3035,7 +3095,7 @@
         <v>6347</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.1522</v>
@@ -3046,16 +3106,19 @@
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
+      <c r="N16" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>44</v>
@@ -3074,7 +3137,7 @@
         <v>17448</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.3896</v>
@@ -3085,16 +3148,19 @@
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
+      <c r="N17" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>44</v>
@@ -3113,7 +3179,7 @@
         <v>359711</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.0689</v>
@@ -3124,16 +3190,19 @@
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
+      <c r="N18" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>58</v>
@@ -3152,7 +3221,7 @@
         <v>604913</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.0116</v>
@@ -3163,16 +3232,19 @@
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
+      <c r="N19" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>6</v>
@@ -3191,7 +3263,7 @@
         <v>6533239</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.0032</v>
@@ -3202,16 +3274,19 @@
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
+      <c r="N20" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>6</v>
@@ -3230,7 +3305,7 @@
         <v>24638739</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.0022</v>
@@ -3241,16 +3316,19 @@
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
+      <c r="N21" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>68</v>
@@ -3269,7 +3347,7 @@
         <v>215344</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.0083</v>
@@ -3280,16 +3358,19 @@
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
+      <c r="N22" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>273</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>269</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>6</v>
@@ -3308,7 +3389,7 @@
         <v>557932</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.0018</v>
@@ -3318,10 +3399,13 @@
         <v>OK</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>275</v>
+        <v>279</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3329,10 +3413,10 @@
         <v>75</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>6</v>
@@ -3351,7 +3435,7 @@
         <v>800608</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.0021</v>
@@ -3362,16 +3446,19 @@
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
+      <c r="N24" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>6</v>
@@ -3390,7 +3477,7 @@
         <v>167333</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.0014</v>
@@ -3400,10 +3487,13 @@
         <v>OK</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>279</v>
+        <v>283</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3411,10 +3501,10 @@
         <v>81</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>6</v>
@@ -3433,7 +3523,7 @@
         <v>25726</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.002</v>
@@ -3443,10 +3533,13 @@
         <v>OK</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3454,10 +3547,10 @@
         <v>84</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>6</v>
@@ -3476,7 +3569,7 @@
         <v>3673590</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.0021</v>
@@ -3487,16 +3580,19 @@
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
+      <c r="N27" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>6</v>
@@ -3515,7 +3611,7 @@
         <v>24070818</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.0015</v>
@@ -3526,16 +3622,19 @@
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
+      <c r="N28" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>6</v>
@@ -3554,7 +3653,7 @@
         <v>8924269</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.0026</v>
@@ -3564,10 +3663,13 @@
         <v>OK</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>288</v>
+        <v>292</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,10 +3677,10 @@
         <v>93</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>6</v>
@@ -3597,7 +3699,7 @@
         <v>1089463</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.0015</v>
@@ -3608,16 +3710,19 @@
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
+      <c r="N30" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
         <v>96</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>6</v>
@@ -3636,7 +3741,7 @@
         <v>7021751</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.0018</v>
@@ -3647,16 +3752,19 @@
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
+      <c r="N31" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
         <v>99</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>6</v>
@@ -3675,7 +3783,7 @@
         <v>2428655</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.0016</v>
@@ -3686,16 +3794,19 @@
       </c>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
+      <c r="N32" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>6</v>
@@ -3714,7 +3825,7 @@
         <v>1155065</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.0011</v>
@@ -3724,10 +3835,13 @@
         <v>OK</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>295</v>
+        <v>299</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3735,10 +3849,10 @@
         <v>105</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>6</v>
@@ -3757,7 +3871,7 @@
         <v>3567540</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.0024</v>
@@ -3768,16 +3882,19 @@
       </c>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
+      <c r="N34" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
         <v>109</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>108</v>
@@ -3796,7 +3913,7 @@
         <v>18813</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.0314</v>
@@ -3807,16 +3924,19 @@
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
+      <c r="N35" s="2" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
         <v>112</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>6</v>
@@ -3835,7 +3955,7 @@
         <v>6148373</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.0026</v>
@@ -3845,10 +3965,13 @@
         <v>OK</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>300</v>
+        <v>304</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3856,13 +3979,13 @@
         <v>116</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>114</v>
@@ -3878,7 +4001,7 @@
         <v>16754</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.6753</v>
@@ -3889,16 +4012,19 @@
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N37" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
         <v>120</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>119</v>
@@ -3917,7 +4043,7 @@
         <v>1850</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.0813</v>
@@ -3928,16 +4054,19 @@
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
-    </row>
-    <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N38" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>124</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>123</v>
@@ -3956,7 +4085,7 @@
         <v>5</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1.295</v>
@@ -3966,10 +4095,13 @@
         <v>SHORT</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>308</v>
+        <v>313</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,10 +4109,10 @@
         <v>128</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>127</v>
@@ -3999,7 +4131,7 @@
         <v>7914</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>2.5362</v>
@@ -4010,16 +4142,19 @@
       </c>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N40" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
         <v>132</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>306</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>131</v>
@@ -4038,7 +4173,7 @@
         <v>1993</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>1.0259</v>
@@ -4049,6 +4184,9 @@
       </c>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
+      <c r="N41" s="2" t="s">
+        <v>318</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>